<commit_message>
feat(bom): show partial subtotals and edit individual prices
</commit_message>
<xml_diff>
--- a/frontend/public/fixtures/ved-synthetic-pricing.xlsx
+++ b/frontend/public/fixtures/ved-synthetic-pricing.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client prices" sheetId="1" r:id="R207b80293f0d4610"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expected results" sheetId="2" r:id="R2fc18a500a5d47c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="3" r:id="R174d2172ccc8422a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client prices" sheetId="1" r:id="R0b6a2495f8eb4dbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expected results" sheetId="2" r:id="R730ee54c43ae416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="3" r:id="Rdf13dddb44384501"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -56,7 +56,7 @@
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -83,6 +83,16 @@
         <x:fgColor rgb="FFE6EAF0"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6EAF0"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF0E8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border>
@@ -96,7 +106,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="20">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -146,6 +156,24 @@
     </x:xf>
     <x:xf numFmtId="201" fontId="6" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -375,7 +403,7 @@
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>Use rows 4–9. Exclude rows 10–13; review reasons. Quantity 999 is reference only.</x:v>
+        <x:v>Synthetic testing only. Upload applies compatible prices automatically. Quantities remain calculated by VED.</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -409,7 +437,7 @@
         <x:v>Quantity</x:v>
       </x:c>
       <x:c r="H3" s="11" t="str">
-        <x:v>Catalog units per purchase</x:v>
+        <x:v>Units per purchase</x:v>
       </x:c>
       <x:c r="I3" s="11" t="str">
         <x:v>Validation note</x:v>
@@ -656,9 +684,7 @@
       <x:c r="D12" s="12" t="str">
         <x:v>piece</x:v>
       </x:c>
-      <x:c r="E12" s="14" t="n">
-        <x:v>65</x:v>
-      </x:c>
+      <x:c r="E12" s="14"/>
       <x:c r="F12" s="12" t="str">
         <x:v>PHP</x:v>
       </x:c>
@@ -669,7 +695,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="I12" s="12" t="str">
-        <x:v>Resolve catalog identity or exclude</x:v>
+        <x:v>Invalid-price fixture; automatically skipped</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
@@ -699,6 +725,195 @@
       </x:c>
       <x:c r="I13" s="12" t="str">
         <x:v>Reject: code is 3.5 mm2; exclude</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="3" t="str">
+        <x:v>DV-LAMP-1X40</x:v>
+      </x:c>
+      <x:c r="B14" s="3" t="str">
+        <x:v>FableVolt 1 x 40 watts fluorescent lamp</x:v>
+      </x:c>
+      <x:c r="C14" s="3" t="str">
+        <x:v>1 x 40 W fluorescent</x:v>
+      </x:c>
+      <x:c r="D14" s="3" t="str">
+        <x:v>piece</x:v>
+      </x:c>
+      <x:c r="E14" s="18" t="n">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="F14" s="3" t="str">
+        <x:v>PHP</x:v>
+      </x:c>
+      <x:c r="G14" s="3"/>
+      <x:c r="H14" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I14" s="3" t="str">
+        <x:v>Synthetic lighting product</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="3" t="str">
+        <x:v>DV-LAMP-2X40</x:v>
+      </x:c>
+      <x:c r="B15" s="3" t="str">
+        <x:v>FableVolt 2 x 40 watts fluorescent lamp</x:v>
+      </x:c>
+      <x:c r="C15" s="3" t="str">
+        <x:v>2 x 40 W fluorescent</x:v>
+      </x:c>
+      <x:c r="D15" s="3" t="str">
+        <x:v>piece</x:v>
+      </x:c>
+      <x:c r="E15" s="18" t="n">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="F15" s="3" t="str">
+        <x:v>PHP</x:v>
+      </x:c>
+      <x:c r="G15" s="3"/>
+      <x:c r="H15" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I15" s="3" t="str">
+        <x:v>Synthetic lighting product</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="3" t="str">
+        <x:v>DV-SWITCH-2</x:v>
+      </x:c>
+      <x:c r="B16" s="3" t="str">
+        <x:v>FableVolt Two gang device switch</x:v>
+      </x:c>
+      <x:c r="C16" s="3" t="str">
+        <x:v>2 gang</x:v>
+      </x:c>
+      <x:c r="D16" s="3" t="str">
+        <x:v>piece</x:v>
+      </x:c>
+      <x:c r="E16" s="18" t="n">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="F16" s="3" t="str">
+        <x:v>PHP</x:v>
+      </x:c>
+      <x:c r="G16" s="3"/>
+      <x:c r="H16" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I16" s="3" t="str">
+        <x:v>Synthetic switch product</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="3" t="str">
+        <x:v>DV-SWITCH-3</x:v>
+      </x:c>
+      <x:c r="B17" s="3" t="str">
+        <x:v>FableVolt Three gang device switch</x:v>
+      </x:c>
+      <x:c r="C17" s="3" t="str">
+        <x:v>3 gang</x:v>
+      </x:c>
+      <x:c r="D17" s="3" t="str">
+        <x:v>piece</x:v>
+      </x:c>
+      <x:c r="E17" s="18" t="n">
+        <x:v>130</x:v>
+      </x:c>
+      <x:c r="F17" s="3" t="str">
+        <x:v>PHP</x:v>
+      </x:c>
+      <x:c r="G17" s="3"/>
+      <x:c r="H17" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I17" s="3" t="str">
+        <x:v>Synthetic switch product</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="3" t="str">
+        <x:v>DV-DOWNLIGHT-200</x:v>
+      </x:c>
+      <x:c r="B18" s="3" t="str">
+        <x:v>FableVolt 200 mm LED recessed downlight</x:v>
+      </x:c>
+      <x:c r="C18" s="3" t="str">
+        <x:v>200 mm LED</x:v>
+      </x:c>
+      <x:c r="D18" s="3" t="str">
+        <x:v>piece</x:v>
+      </x:c>
+      <x:c r="E18" s="18" t="n">
+        <x:v>350</x:v>
+      </x:c>
+      <x:c r="F18" s="3" t="str">
+        <x:v>PHP</x:v>
+      </x:c>
+      <x:c r="G18" s="3"/>
+      <x:c r="H18" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I18" s="3" t="str">
+        <x:v>Synthetic lighting product</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="64" customHeight="1">
+      <x:c r="A19" s="3" t="str">
+        <x:v>DV-OUTLET-10</x:v>
+      </x:c>
+      <x:c r="B19" s="3" t="str">
+        <x:v>FableVolt Duplex convenience outlet grounding type 10 amps 250 volt with modern plate cover</x:v>
+      </x:c>
+      <x:c r="C19" s="3" t="str">
+        <x:v>10 A 250 V duplex</x:v>
+      </x:c>
+      <x:c r="D19" s="3" t="str">
+        <x:v>piece</x:v>
+      </x:c>
+      <x:c r="E19" s="18" t="n">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="F19" s="3" t="str">
+        <x:v>PHP</x:v>
+      </x:c>
+      <x:c r="G19" s="3"/>
+      <x:c r="H19" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I19" s="3" t="str">
+        <x:v>Synthetic power product</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="3" t="str">
+        <x:v>DV-PANEL</x:v>
+      </x:c>
+      <x:c r="B20" s="3" t="str">
+        <x:v>FableVolt Panelboard</x:v>
+      </x:c>
+      <x:c r="C20" s="3" t="str">
+        <x:v>Panelboard</x:v>
+      </x:c>
+      <x:c r="D20" s="3" t="str">
+        <x:v>piece</x:v>
+      </x:c>
+      <x:c r="E20" s="18" t="n">
+        <x:v>1200</x:v>
+      </x:c>
+      <x:c r="F20" s="3" t="str">
+        <x:v>PHP</x:v>
+      </x:c>
+      <x:c r="G20" s="3"/>
+      <x:c r="H20" s="3" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I20" s="3" t="str">
+        <x:v>Synthetic panel product</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -882,6 +1097,111 @@
       <x:c r="C13" s="3"/>
       <x:c r="D13" s="3"/>
     </x:row>
+    <x:row r="15" ht="36" customHeight="1">
+      <x:c r="A15" s="20" t="str">
+        <x:v>Lighting plan test</x:v>
+      </x:c>
+      <x:c r="B15" s="20"/>
+      <x:c r="C15" s="20"/>
+      <x:c r="D15" s="20"/>
+    </x:row>
+    <x:row r="16" ht="36" customHeight="1">
+      <x:c r="A16" s="21" t="str">
+        <x:v>Device</x:v>
+      </x:c>
+      <x:c r="B16" s="21" t="str">
+        <x:v>Quantity</x:v>
+      </x:c>
+      <x:c r="C16" s="21" t="str">
+        <x:v>PHP per piece</x:v>
+      </x:c>
+      <x:c r="D16" s="21" t="str">
+        <x:v>Expected PHP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="36" customHeight="1">
+      <x:c r="A17" s="20" t="str">
+        <x:v>1 x 40 watts fluorescent lamp</x:v>
+      </x:c>
+      <x:c r="B17" s="20" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="C17" s="24" t="n">
+        <x:f>'Client prices'!E14</x:f>
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="D17" s="24" t="n">
+        <x:f>B17*C17</x:f>
+        <x:v>1800</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="36" customHeight="1">
+      <x:c r="A18" s="20" t="str">
+        <x:v>2 x 40 watts fluorescent lamp</x:v>
+      </x:c>
+      <x:c r="B18" s="20" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="C18" s="24" t="n">
+        <x:f>'Client prices'!E15</x:f>
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="D18" s="24" t="n">
+        <x:f>B18*C18</x:f>
+        <x:v>12000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="36" customHeight="1">
+      <x:c r="A19" s="20" t="str">
+        <x:v>One gang device switch</x:v>
+      </x:c>
+      <x:c r="B19" s="20" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C19" s="24" t="n">
+        <x:f>'Client prices'!E5</x:f>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="D19" s="24" t="n">
+        <x:f>B19*C19</x:f>
+        <x:v>360</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="36" customHeight="1">
+      <x:c r="A20" s="20" t="str">
+        <x:v>Two gang device switch</x:v>
+      </x:c>
+      <x:c r="B20" s="20" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="C20" s="24" t="n">
+        <x:f>'Client prices'!E16</x:f>
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="D20" s="24" t="n">
+        <x:f>B20*C20</x:f>
+        <x:v>285</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="36" customHeight="1">
+      <x:c r="A21" s="23" t="str">
+        <x:v>Known device subtotal</x:v>
+      </x:c>
+      <x:c r="B21" s="23"/>
+      <x:c r="C21" s="25"/>
+      <x:c r="D21" s="25" t="n">
+        <x:f>SUM(D17:D20)</x:f>
+        <x:v>14445</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="36" customHeight="1">
+      <x:c r="A22" s="20" t="str">
+        <x:v>Wire/conduit quantities are calculated by VED.</x:v>
+      </x:c>
+      <x:c r="B22" s="20"/>
+      <x:c r="C22" s="20"/>
+      <x:c r="D22" s="20"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -912,74 +1232,74 @@
     </x:row>
     <x:row r="2" ht="48" customHeight="1">
       <x:c r="A2" s="3" t="str">
-        <x:v>1 · Start fixture</x:v>
+        <x:v>Upload</x:v>
       </x:c>
       <x:c r="B2" s="3" t="str">
-        <x:v>Run scripts/serve_synthetic_pricing_fixture.py against the empty restricted verification database.</x:v>
+        <x:v>Choose this workbook using Upload BOM. Prices apply automatically to compatible existing items.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>2 · Upload</x:v>
+        <x:v>Scope</x:v>
       </x:c>
       <x:c r="B3" s="3" t="str">
-        <x:v>Open the printed Cost estimation URL. Choose this workbook using Upload BOM.</x:v>
+        <x:v>Workspace upload affects the current floor. Cost estimation upload affects the project.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="48" customHeight="1">
       <x:c r="A4" s="3" t="str">
-        <x:v>3 · Map</x:v>
+        <x:v>Edit</x:v>
       </x:c>
       <x:c r="B4" s="3" t="str">
-        <x:v>Exclude Client prices:10 through Client prices:13, then Check mappings and Use imported prices.</x:v>
+        <x:v>Use Edit prices to override an individual device, wire/cable or conduit price.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="48" customHeight="1">
       <x:c r="A5" s="3" t="str">
-        <x:v>4 · Devices</x:v>
+        <x:v>Quantities</x:v>
       </x:c>
       <x:c r="B5" s="3" t="str">
-        <x:v>Select imported outlet and switch prices. Select visible results, preview and apply.</x:v>
+        <x:v>Client quantities never replace the calculated takeoff.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
       <x:c r="A6" s="3" t="str">
-        <x:v>5 · Path A</x:v>
+        <x:v>Lighting test</x:v>
       </x:c>
       <x:c r="B6" s="3" t="str">
-        <x:v>Choose THHN 3.5 mm2 and PVC 20 mm for canonical:1.</x:v>
+        <x:v>The shown 4 single lamps, 16 twin lamps, 6 one-gang and 3 two-gang switches total PHP 14,445.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="48" customHeight="1">
       <x:c r="A7" s="3" t="str">
-        <x:v>6 · Path B</x:v>
+        <x:v>Wire and conduit</x:v>
       </x:c>
       <x:c r="B7" s="3" t="str">
-        <x:v>Choose 2C cable and EMT 20 mm for canonical:2.</x:v>
+        <x:v>Each path has separate cable and conduit components. Conversions are explicit.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="48" customHeight="1">
       <x:c r="A8" s="3" t="str">
-        <x:v>7 · Apply</x:v>
+        <x:v>Invalid examples</x:v>
       </x:c>
       <x:c r="B8" s="3" t="str">
-        <x:v>Preview selected or all compatible existing wiring paths. Apply, Finish, then reload.</x:v>
+        <x:v>Original invalid-price and conflicting-code rows remain parser examples and are skipped.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="48" customHeight="1">
       <x:c r="A9" s="3" t="str">
-        <x:v>8 · Validate</x:v>
+        <x:v>Synthetic only</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>Expected priced subtotal PHP 980. Prices are per measured metre after explicit conversion.</x:v>
+        <x:v>Fictional prices and products, not a client quote or an approved specification.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
       <x:c r="A10" s="3" t="str">
-        <x:v>9 · Cleanup</x:v>
+        <x:v>Missing heights</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>Stop the isolated fixture with Ctrl+C. Only its exact test records are removed; real projects are untouched.</x:v>
+        <x:v>Known horizontal costs can be partial. Actual drops require stored service and mounting heights.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>